<commit_message>
feat : thêm button xettuyen báo Trúng/rớt
</commit_message>
<xml_diff>
--- a/excel_imports/Quan ly nganh.xlsx
+++ b/excel_imports/Quan ly nganh.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="110">
   <si>
     <t>Mã ngành</t>
   </si>
@@ -77,60 +77,96 @@
     <t>D01</t>
   </si>
   <si>
+    <t>22.59</t>
+  </si>
+  <si>
     <t>Giáo dục mầm non</t>
   </si>
   <si>
     <t>M01</t>
   </si>
   <si>
+    <t>24.2</t>
+  </si>
+  <si>
     <t>Giáo dục Tiểu học</t>
   </si>
   <si>
+    <t>25.12</t>
+  </si>
+  <si>
     <t>Giáo dục Chính trị</t>
   </si>
   <si>
+    <t>24.04</t>
+  </si>
+  <si>
     <t>Sư phạm Toán học</t>
   </si>
   <si>
     <t>A01</t>
   </si>
   <si>
+    <t>27.21</t>
+  </si>
+  <si>
     <t>Sư phạm Vật lý</t>
   </si>
   <si>
+    <t>27.64</t>
+  </si>
+  <si>
     <t>Sư phạm Hoá học</t>
   </si>
   <si>
     <t>D07</t>
   </si>
   <si>
+    <t>27.36</t>
+  </si>
+  <si>
     <t>Sư phạm Sinh học</t>
   </si>
   <si>
     <t>B08</t>
   </si>
   <si>
+    <t>24.77</t>
+  </si>
+  <si>
     <t>Sư phạm Ngữ văn</t>
   </si>
   <si>
+    <t>24.96</t>
+  </si>
+  <si>
     <t>Sư phạm Lịch sử</t>
   </si>
   <si>
     <t>D14</t>
   </si>
   <si>
+    <t>28.39</t>
+  </si>
+  <si>
     <t>Sư phạm Địa lý</t>
   </si>
   <si>
     <t>D15</t>
   </si>
   <si>
+    <t>28.55</t>
+  </si>
+  <si>
     <t>Sư phạm Âm nhạc</t>
   </si>
   <si>
     <t>N01</t>
   </si>
   <si>
+    <t>22.0</t>
+  </si>
+  <si>
     <t>Sư phạm Mỹ thuật</t>
   </si>
   <si>
@@ -140,91 +176,163 @@
     <t>Sư phạm Tiếng Anh</t>
   </si>
   <si>
+    <t>27.18</t>
+  </si>
+  <si>
     <t>Sư phạm khoa học tự nhiên</t>
   </si>
   <si>
+    <t>24.86</t>
+  </si>
+  <si>
     <t>Sư phạm Lịch sử - Địa lí</t>
   </si>
   <si>
     <t>Ngôn ngữ Anh</t>
   </si>
   <si>
+    <t>24.79</t>
+  </si>
+  <si>
     <t>Lịch sử</t>
   </si>
   <si>
+    <t>27.02</t>
+  </si>
+  <si>
     <t>Tâm lý học</t>
   </si>
   <si>
+    <t>22.25</t>
+  </si>
+  <si>
     <t>Địa lý học</t>
   </si>
   <si>
+    <t>26.84</t>
+  </si>
+  <si>
     <t>Quốc tế học</t>
   </si>
   <si>
+    <t>21.0</t>
+  </si>
+  <si>
     <t>Việt Nam học</t>
   </si>
   <si>
     <t xml:space="preserve">Thông tin - thư viện </t>
   </si>
   <si>
+    <t>26.48</t>
+  </si>
+  <si>
     <t>Quản trị kinh doanh</t>
   </si>
   <si>
+    <t>20.24</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kinh doanh quốc tế </t>
   </si>
   <si>
+    <t>21.3</t>
+  </si>
+  <si>
     <t>Tài chính – Ngân hàng</t>
   </si>
   <si>
     <t>Kế toán</t>
   </si>
   <si>
+    <t>19.94</t>
+  </si>
+  <si>
     <t>Kiểm toán</t>
   </si>
   <si>
+    <t>21.7</t>
+  </si>
+  <si>
     <t>Quản trị văn phòng</t>
   </si>
   <si>
     <t>Luật</t>
   </si>
   <si>
+    <t>21.58</t>
+  </si>
+  <si>
     <t>Khoa học môi trường</t>
   </si>
   <si>
+    <t>19.24</t>
+  </si>
+  <si>
     <t>Khoa học dữ liệu</t>
   </si>
   <si>
+    <t>22.05</t>
+  </si>
+  <si>
     <t>Toán ứng dụng</t>
   </si>
   <si>
+    <t>23.85</t>
+  </si>
+  <si>
     <t>Kỹ thuật phần mềm</t>
   </si>
   <si>
+    <t>20.99</t>
+  </si>
+  <si>
     <t>Trí tuệ nhân tạo</t>
   </si>
   <si>
+    <t>21.99</t>
+  </si>
+  <si>
     <t>Công nghệ thông tin</t>
   </si>
   <si>
     <t>Công nghệ kỹ thuật điện, điện tử</t>
   </si>
   <si>
+    <t>21.54</t>
+  </si>
+  <si>
     <t>Công nghệ kỹ thuật điện tử - viễn thông</t>
   </si>
   <si>
     <t>Công nghệ kỹ thuật môi trường</t>
   </si>
   <si>
+    <t>18.95</t>
+  </si>
+  <si>
     <t>Kỹ thuật điện</t>
   </si>
   <si>
+    <t>19.93</t>
+  </si>
+  <si>
     <t>Kỹ thuật điện tử - viễn thông</t>
   </si>
   <si>
+    <t>19.96</t>
+  </si>
+  <si>
     <t>Du lịch</t>
   </si>
   <si>
+    <t>21.95</t>
+  </si>
+  <si>
     <t>Quản trị nhà hàng và dịch vụ ăn uống</t>
+  </si>
+  <si>
+    <t>20.83</t>
   </si>
   <si>
     <t>7220201CLC</t>
@@ -261,7 +369,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -301,23 +409,29 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -464,7 +578,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -479,6 +593,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFAFAFA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -664,7 +784,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -684,6 +804,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFEBEBEB"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFEBEBEB"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFEBEBEB"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFEBEBEB"/>
       </bottom>
       <diagonal/>
     </border>
@@ -788,70 +923,67 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -866,74 +998,77 @@
     <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -967,13 +1102,18 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1399,22 +1539,28 @@
       <c r="E2" s="12">
         <v>17</v>
       </c>
+      <c r="F2" s="13" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="3" ht="20.25" customHeight="1" spans="1:14">
       <c r="A3" s="9">
         <v>7140201</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="12">
         <v>200</v>
       </c>
       <c r="E3" s="12">
         <v>20</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="4" ht="20.25" customHeight="1" spans="1:14">
@@ -1422,7 +1568,7 @@
         <v>7140202</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>15</v>
@@ -1431,6 +1577,9 @@
         <v>200</v>
       </c>
       <c r="E4" s="12">
+        <v>21</v>
+      </c>
+      <c r="F4" s="13" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1439,7 +1588,7 @@
         <v>7140205</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>15</v>
@@ -1448,6 +1597,9 @@
         <v>10</v>
       </c>
       <c r="E5" s="12">
+        <v>23</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1456,16 +1608,19 @@
         <v>7140209</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D6" s="12">
         <v>40</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="14">
         <v>24.5</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="7" ht="20.25" customHeight="1" spans="1:14">
@@ -1473,16 +1628,19 @@
         <v>7140211</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D7" s="12">
         <v>10</v>
       </c>
       <c r="E7" s="12">
         <v>24</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="8" ht="20.25" customHeight="1" spans="1:14">
@@ -1490,10 +1648,10 @@
         <v>7140212</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D8" s="12">
         <v>10</v>
@@ -1501,22 +1659,29 @@
       <c r="E8" s="12">
         <v>24</v>
       </c>
+      <c r="F8" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="15"/>
     </row>
     <row r="9" ht="20.25" customHeight="1" spans="1:14">
       <c r="A9" s="9">
         <v>7140213</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="D9" s="12">
         <v>10</v>
       </c>
       <c r="E9" s="12">
         <v>23</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="10" ht="20.25" customHeight="1" spans="1:14">
@@ -1524,7 +1689,7 @@
         <v>7140217</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>15</v>
@@ -1534,6 +1699,9 @@
       </c>
       <c r="E10" s="12">
         <v>24</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="11" ht="20.25" customHeight="1" spans="1:14">
@@ -1541,16 +1709,19 @@
         <v>7140218</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D11" s="12">
         <v>10</v>
       </c>
       <c r="E11" s="12">
         <v>25</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="12" ht="20.25" customHeight="1" spans="1:14">
@@ -1558,16 +1729,19 @@
         <v>7140219</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="D12" s="12">
         <v>10</v>
       </c>
       <c r="E12" s="12">
         <v>25</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="13" ht="20.25" customHeight="1" spans="1:14">
@@ -1575,16 +1749,19 @@
         <v>7140221</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D13" s="12">
         <v>75</v>
       </c>
       <c r="E13" s="12">
         <v>18</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="14" ht="20.25" customHeight="1" spans="1:14">
@@ -1592,16 +1769,19 @@
         <v>7140222</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="D14" s="12">
         <v>75</v>
       </c>
       <c r="E14" s="12">
         <v>18</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="15" ht="20.25" customHeight="1" spans="1:14">
@@ -1609,16 +1789,19 @@
         <v>7140231</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D15" s="12">
         <v>120</v>
       </c>
       <c r="E15" s="12">
         <v>24</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="16" ht="20.25" customHeight="1" spans="1:14">
@@ -1626,10 +1809,10 @@
         <v>7140247</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D16" s="12">
         <v>60</v>
@@ -1637,16 +1820,19 @@
       <c r="E16" s="12">
         <v>22</v>
       </c>
-    </row>
-    <row r="17" ht="20.25" customHeight="1" spans="1:5">
+      <c r="F16" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" ht="20.25" customHeight="1" spans="1:6">
       <c r="A17" s="9">
         <v>7140249</v>
       </c>
       <c r="B17" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>38</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>29</v>
       </c>
       <c r="D17" s="12">
         <v>40</v>
@@ -1654,16 +1840,19 @@
       <c r="E17" s="12">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" ht="20.25" customHeight="1" spans="1:5">
+      <c r="F17" s="16">
+        <v>28.39</v>
+      </c>
+    </row>
+    <row r="18" ht="20.25" customHeight="1" spans="1:6">
       <c r="A18" s="9">
         <v>7220201</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D18" s="12">
         <v>260</v>
@@ -1671,16 +1860,19 @@
       <c r="E18" s="12">
         <v>22</v>
       </c>
-    </row>
-    <row r="19" ht="20.25" customHeight="1" spans="1:5">
+      <c r="F18" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" ht="20.25" customHeight="1" spans="1:6">
       <c r="A19" s="9">
         <v>7229010</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D19" s="12">
         <v>30</v>
@@ -1688,13 +1880,16 @@
       <c r="E19" s="12">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" ht="20.25" customHeight="1" spans="1:5">
+      <c r="F19" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" ht="20.25" customHeight="1" spans="1:6">
       <c r="A20" s="9">
         <v>7310401</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>15</v>
@@ -1705,16 +1900,19 @@
       <c r="E20" s="12">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" ht="20.25" customHeight="1" spans="1:5">
+      <c r="F20" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" ht="20.25" customHeight="1" spans="1:6">
       <c r="A21" s="9">
         <v>7310501</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="D21" s="12">
         <v>30</v>
@@ -1722,13 +1920,16 @@
       <c r="E21" s="12">
         <v>17</v>
       </c>
-    </row>
-    <row r="22" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F21" s="13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" ht="18.75" customHeight="1" spans="1:6">
       <c r="A22" s="9">
         <v>7310601</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>15</v>
@@ -1739,13 +1940,16 @@
       <c r="E22" s="12">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F22" s="13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" ht="18.75" customHeight="1" spans="1:6">
       <c r="A23" s="9">
         <v>7310630</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>15</v>
@@ -1756,13 +1960,16 @@
       <c r="E23" s="12">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F23" s="13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" ht="18.75" customHeight="1" spans="1:6">
       <c r="A24" s="9">
         <v>7320201</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>15</v>
@@ -1773,98 +1980,116 @@
       <c r="E24" s="12">
         <v>17</v>
       </c>
-    </row>
-    <row r="25" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F24" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" ht="18.75" customHeight="1" spans="1:6">
       <c r="A25" s="9">
         <v>7340101</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D25" s="12">
         <v>360</v>
       </c>
-      <c r="E25" s="13">
+      <c r="E25" s="14">
         <v>18.5</v>
       </c>
-    </row>
-    <row r="26" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F25" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="26" ht="18.75" customHeight="1" spans="1:6">
       <c r="A26" s="9">
         <v>7340120</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D26" s="12">
         <v>200</v>
       </c>
-      <c r="E26" s="13">
+      <c r="E26" s="14">
         <v>18.5</v>
       </c>
-    </row>
-    <row r="27" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F26" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" ht="18.75" customHeight="1" spans="1:6">
       <c r="A27" s="9">
         <v>7340201</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D27" s="12">
         <v>500</v>
       </c>
-      <c r="E27" s="13">
+      <c r="E27" s="14">
         <v>18.5</v>
       </c>
-    </row>
-    <row r="28" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F27" s="13">
+        <v>19.48</v>
+      </c>
+    </row>
+    <row r="28" ht="18.75" customHeight="1" spans="1:6">
       <c r="A28" s="9">
         <v>7340301</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D28" s="12">
         <v>380</v>
       </c>
-      <c r="E28" s="13">
+      <c r="E28" s="14">
         <v>18.5</v>
       </c>
-    </row>
-    <row r="29" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F28" s="13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" ht="18.75" customHeight="1" spans="1:6">
       <c r="A29" s="9">
         <v>7340302</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D29" s="12">
         <v>60</v>
       </c>
-      <c r="E29" s="13">
+      <c r="E29" s="14">
         <v>18.5</v>
       </c>
-    </row>
-    <row r="30" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F29" s="13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" ht="18.75" customHeight="1" spans="1:6">
       <c r="A30" s="9">
         <v>7340406</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>15</v>
@@ -1875,13 +2100,16 @@
       <c r="E30" s="12">
         <v>17</v>
       </c>
-    </row>
-    <row r="31" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F30" s="13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" ht="18.75" customHeight="1" spans="1:6">
       <c r="A31" s="9">
         <v>7380101</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>15</v>
@@ -1892,16 +2120,19 @@
       <c r="E31" s="12">
         <v>17</v>
       </c>
-    </row>
-    <row r="32" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F31" s="13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" ht="18.75" customHeight="1" spans="1:6">
       <c r="A32" s="9">
         <v>7440301</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D32" s="12">
         <v>30</v>
@@ -1909,16 +2140,19 @@
       <c r="E32" s="12">
         <v>18</v>
       </c>
-    </row>
-    <row r="33" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F32" s="13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" ht="18.75" customHeight="1" spans="1:6">
       <c r="A33" s="9">
         <v>7460108</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D33" s="12">
         <v>80</v>
@@ -1926,16 +2160,19 @@
       <c r="E33" s="12">
         <v>21</v>
       </c>
-    </row>
-    <row r="34" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F33" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" ht="18.75" customHeight="1" spans="1:6">
       <c r="A34" s="9">
         <v>7460112</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D34" s="12">
         <v>90</v>
@@ -1943,16 +2180,19 @@
       <c r="E34" s="12">
         <v>22</v>
       </c>
-    </row>
-    <row r="35" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F34" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" ht="18.75" customHeight="1" spans="1:6">
       <c r="A35" s="9">
         <v>7480103</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>56</v>
+        <v>84</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D35" s="12">
         <v>110</v>
@@ -1960,16 +2200,19 @@
       <c r="E35" s="12">
         <v>21</v>
       </c>
-    </row>
-    <row r="36" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F35" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" ht="18.75" customHeight="1" spans="1:6">
       <c r="A36" s="9">
         <v>7480107</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D36" s="12">
         <v>80</v>
@@ -1977,16 +2220,19 @@
       <c r="E36" s="12">
         <v>22</v>
       </c>
-    </row>
-    <row r="37" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F36" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="37" ht="18.75" customHeight="1" spans="1:6">
       <c r="A37" s="9">
         <v>7480201</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>58</v>
+        <v>88</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D37" s="12">
         <v>400</v>
@@ -1994,16 +2240,19 @@
       <c r="E37" s="12">
         <v>21</v>
       </c>
-    </row>
-    <row r="38" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F37" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="38" ht="18.75" customHeight="1" spans="1:6">
       <c r="A38" s="9">
         <v>7510301</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D38" s="12">
         <v>45</v>
@@ -2011,16 +2260,19 @@
       <c r="E38" s="12">
         <v>18</v>
       </c>
-    </row>
-    <row r="39" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F38" s="13" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="39" ht="18.75" customHeight="1" spans="1:6">
       <c r="A39" s="9">
         <v>7510302</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D39" s="12">
         <v>45</v>
@@ -2028,16 +2280,19 @@
       <c r="E39" s="12">
         <v>18</v>
       </c>
-    </row>
-    <row r="40" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F39" s="13">
+        <v>20.25</v>
+      </c>
+    </row>
+    <row r="40" ht="18.75" customHeight="1" spans="1:6">
       <c r="A40" s="9">
         <v>7510406</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>61</v>
+        <v>92</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D40" s="12">
         <v>30</v>
@@ -2045,16 +2300,19 @@
       <c r="E40" s="12">
         <v>18</v>
       </c>
-    </row>
-    <row r="41" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F40" s="13" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="41" ht="18.75" customHeight="1" spans="1:6">
       <c r="A41" s="9">
         <v>7520201</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D41" s="12">
         <v>30</v>
@@ -2062,16 +2320,19 @@
       <c r="E41" s="12">
         <v>18</v>
       </c>
-    </row>
-    <row r="42" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F41" s="13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="42" ht="18.75" customHeight="1" spans="1:6">
       <c r="A42" s="9">
         <v>7520207</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D42" s="12">
         <v>90</v>
@@ -2079,13 +2340,16 @@
       <c r="E42" s="12">
         <v>19</v>
       </c>
-    </row>
-    <row r="43" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F42" s="13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="43" ht="18.75" customHeight="1" spans="1:6">
       <c r="A43" s="9">
         <v>7810101</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>15</v>
@@ -2093,19 +2357,22 @@
       <c r="D43" s="12">
         <v>120</v>
       </c>
-      <c r="E43" s="13">
+      <c r="E43" s="14">
         <v>20.5</v>
       </c>
-    </row>
-    <row r="44" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F43" s="13" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="44" ht="18.75" customHeight="1" spans="1:6">
       <c r="A44" s="9">
         <v>7810202</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D44" s="12">
         <v>60</v>
@@ -2113,16 +2380,19 @@
       <c r="E44" s="12">
         <v>18</v>
       </c>
-    </row>
-    <row r="45" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F44" s="13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" ht="18.75" customHeight="1" spans="1:6">
       <c r="A45" s="9" t="s">
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D45" s="12">
         <v>100</v>
@@ -2130,50 +2400,59 @@
       <c r="E45" s="12">
         <v>22</v>
       </c>
-    </row>
-    <row r="46" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F45" s="13">
+        <v>23.62</v>
+      </c>
+    </row>
+    <row r="46" ht="18.75" customHeight="1" spans="1:6">
       <c r="A46" s="9" t="s">
-        <v>68</v>
+        <v>104</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D46" s="12">
         <v>100</v>
       </c>
-      <c r="E46" s="13">
+      <c r="E46" s="14">
         <v>18.5</v>
       </c>
-    </row>
-    <row r="47" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F46" s="13">
+        <v>20.62</v>
+      </c>
+    </row>
+    <row r="47" ht="18.75" customHeight="1" spans="1:6">
       <c r="A47" s="9" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D47" s="12">
         <v>50</v>
       </c>
-      <c r="E47" s="13">
+      <c r="E47" s="14">
         <v>18.5</v>
       </c>
-    </row>
-    <row r="48" ht="18.75" customHeight="1" spans="1:5">
+      <c r="F47" s="13">
+        <v>19.25</v>
+      </c>
+    </row>
+    <row r="48" ht="18.75" customHeight="1" spans="1:6">
       <c r="A48" s="9" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D48" s="12">
         <v>350</v>
@@ -2181,20 +2460,23 @@
       <c r="E48" s="12">
         <v>21</v>
       </c>
+      <c r="F48" s="13">
+        <v>22.63</v>
+      </c>
     </row>
     <row r="49" ht="18.75" customHeight="1" spans="1:5">
       <c r="A49" s="9"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="15"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="17"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
     </row>
     <row r="50" ht="18.75" customHeight="1" spans="1:5">
       <c r="A50" s="9"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="15"/>
-      <c r="E50" s="15"/>
+      <c r="B50" s="17"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>